<commit_message>
Data-request sheet: drop 3D-model equipment rows from ③
The equipment in the 3D model is still being built, so ③ is now an
empty input table with a generic example row. Only ⑦ keeps pre-filled
values, which come from the position logs themselves.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLbqDTGA3XkGmHcdVgiZ3k
</commit_message>
<xml_diff>
--- a/flowlab-v6-guide/data-request/生産量推計_データご提供のお願い.xlsx
+++ b/flowlab-v6-guide/data-request/生産量推計_データご提供のお願い.xlsx
@@ -333,7 +333,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">T-203</t>
+          <t xml:space="preserve">No.1</t>
         </r>
         <r>
           <rPr>
@@ -341,23 +341,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">、</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">SS-2000</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">充填ライン </t>
+          <t xml:space="preserve">、充填ライン </t>
         </r>
         <r>
           <rPr>
@@ -673,7 +657,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">実際の設備名・台数の違いなど</t>
+          <t xml:space="preserve">台数・更新予定など</t>
         </r>
       </text>
     </comment>
@@ -819,39 +803,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">例：調合槽 </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">T-203</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">〜</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">220</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">、原料の投入</t>
+          <t xml:space="preserve">例：調合槽、原料の投入</t>
         </r>
       </text>
     </comment>
@@ -872,7 +824,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="207">
   <si>
     <t xml:space="preserve">生産量の推計に向けた データご提供のお願い</t>
   </si>
@@ -1084,7 +1036,7 @@
     <t xml:space="preserve">色の意味</t>
   </si>
   <si>
-    <t xml:space="preserve">黄色＝記入欄　灰色＝記入例　緑＝自動計算　青＝こちらで仮に入れた値（違っていれば上書き）</t>
+    <t xml:space="preserve">黄色＝記入欄　灰色＝記入例　緑＝自動計算　青＝位置ログなど、こちらで記入済みの値（違っていれば上書き）</t>
   </si>
   <si>
     <t xml:space="preserve">シート一覧と記入状況</t>
@@ -1338,7 +1290,7 @@
     <t xml:space="preserve">以前いただいた生産量・販売数・出荷数・金額が、どの期間・単位・細かさかを確認させてください。これで、推計にそのまま使えるかが分かります。</t>
   </si>
   <si>
-    <t xml:space="preserve">黄色＝記入欄（分かる範囲で・空欄可）　灰色＝記入例　緑＝自動計算　青＝こちらで仮に入れた値（違っていれば上書きしてください）</t>
+    <t xml:space="preserve">黄色＝記入欄（分かる範囲で・空欄可）　灰色＝記入例　緑＝自動計算　青＝位置ログなど、こちらで記入済みの値（違っていれば上書きしてください）</t>
   </si>
   <si>
     <t xml:space="preserve">データ</t>
@@ -1803,26 +1755,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">バッチ）でどれだけ・何分で処理できるか。工程ごとの能力と、どこが詰まるか（律速工程）を出すのに使います。青い行は</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF6F8077"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3D</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF6F8077"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">モデルで想定している設備（推定）です。違っていれば直し、足りなければ追加してください。</t>
+      <t xml:space="preserve">バッチ）でどれだけ・何分で処理できるか。工程ごとの能力と、どこが詰まるか（律速工程）を出すのに使います。設備台帳・作業標準書の添付でも構いません。</t>
     </r>
   </si>
   <si>
@@ -1980,7 +1913,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">T-203</t>
+      <t xml:space="preserve">No.1</t>
     </r>
   </si>
   <si>
@@ -2059,498 +1992,6 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">回</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">第一ペイント工場</t>
-  </si>
-  <si>
-    <t xml:space="preserve">分散</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ATOM'X</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">分散ミル </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">M-1</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ATOM'X</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">分散ミル </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">M-2</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ATOM'X</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">分散ミル </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">M-3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ディスパー槽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">T-41</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ディスパー槽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">T-43</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ディスパー槽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">T-47</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ディスパー槽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">T-48</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">調合槽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">T-203</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">調合槽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">T-208</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">調合槽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">T-220</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">貯槽</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KV</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">タンク </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KV-2</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KV</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">タンク </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KV-4</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KV</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">タンク </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KV-6</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KV</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">タンク </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KV-8</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">充填</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SS-2000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">充填ライン </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SS-2000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">充填ライン </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KOYO</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">缶充填機</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">ワニス工場</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ワニス</t>
-  </si>
-  <si>
-    <t xml:space="preserve">調色工場</t>
-  </si>
-  <si>
-    <t xml:space="preserve">第二ペイント工場</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="游ゴシック"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2B</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1C2B25"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（第二・中ロット仕込み）</t>
     </r>
   </si>
   <si>
@@ -2922,6 +2363,9 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
+    <t xml:space="preserve">ワニス</t>
+  </si>
+  <si>
     <t xml:space="preserve">7/24, 7/27, 7/28</t>
   </si>
   <si>
@@ -2958,6 +2402,9 @@
     <t xml:space="preserve">7</t>
   </si>
   <si>
+    <t xml:space="preserve">充填</t>
+  </si>
+  <si>
     <t xml:space="preserve">8/27, 8/28, 8/31</t>
   </si>
   <si>
@@ -2965,6 +2412,27 @@
   </si>
   <si>
     <t xml:space="preserve">9</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1C2B25"/>
+        <rFont val="游ゴシック"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1C2B25"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（第二・中ロット仕込み）</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">8/24, 8/25, 8/26</t>
@@ -3420,10 +2888,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3437,6 +2901,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -13308,15 +12776,9 @@
       <c r="O5" s="26"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="C6" s="35" t="s">
-        <v>128</v>
-      </c>
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
       <c r="F6" s="22"/>
@@ -13331,15 +12793,9 @@
       <c r="O6" s="22"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="C7" s="35" t="s">
-        <v>129</v>
-      </c>
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
       <c r="F7" s="22"/>
@@ -13354,15 +12810,9 @@
       <c r="O7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>130</v>
-      </c>
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
       <c r="D8" s="22"/>
       <c r="E8" s="22"/>
       <c r="F8" s="22"/>
@@ -13377,15 +12827,9 @@
       <c r="O8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>131</v>
-      </c>
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
       <c r="D9" s="22"/>
       <c r="E9" s="22"/>
       <c r="F9" s="22"/>
@@ -13400,15 +12844,9 @@
       <c r="O9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>132</v>
-      </c>
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
       <c r="D10" s="22"/>
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
@@ -13423,15 +12861,9 @@
       <c r="O10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>133</v>
-      </c>
+      <c r="A11" s="22"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
       <c r="D11" s="22"/>
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
@@ -13446,15 +12878,9 @@
       <c r="O11" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="C12" s="21" t="s">
-        <v>134</v>
-      </c>
+      <c r="A12" s="22"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
       <c r="D12" s="22"/>
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
@@ -13469,15 +12895,9 @@
       <c r="O12" s="22"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>135</v>
-      </c>
+      <c r="A13" s="22"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
       <c r="D13" s="22"/>
       <c r="E13" s="22"/>
       <c r="F13" s="22"/>
@@ -13492,15 +12912,9 @@
       <c r="O13" s="22"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="C14" s="21" t="s">
-        <v>136</v>
-      </c>
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
       <c r="D14" s="22"/>
       <c r="E14" s="22"/>
       <c r="F14" s="22"/>
@@ -13515,15 +12929,9 @@
       <c r="O14" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>137</v>
-      </c>
+      <c r="A15" s="22"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
       <c r="D15" s="22"/>
       <c r="E15" s="22"/>
       <c r="F15" s="22"/>
@@ -13538,15 +12946,9 @@
       <c r="O15" s="22"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B16" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="C16" s="35" t="s">
-        <v>139</v>
-      </c>
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
       <c r="D16" s="22"/>
       <c r="E16" s="22"/>
       <c r="F16" s="22"/>
@@ -13561,15 +12963,9 @@
       <c r="O16" s="22"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B17" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="C17" s="35" t="s">
-        <v>140</v>
-      </c>
+      <c r="A17" s="22"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
       <c r="D17" s="22"/>
       <c r="E17" s="22"/>
       <c r="F17" s="22"/>
@@ -13584,15 +12980,9 @@
       <c r="O17" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B18" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="C18" s="35" t="s">
-        <v>141</v>
-      </c>
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
       <c r="D18" s="22"/>
       <c r="E18" s="22"/>
       <c r="F18" s="22"/>
@@ -13607,15 +12997,9 @@
       <c r="O18" s="22"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B19" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="C19" s="35" t="s">
-        <v>142</v>
-      </c>
+      <c r="A19" s="22"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
       <c r="D19" s="22"/>
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
@@ -13630,15 +13014,9 @@
       <c r="O19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="C20" s="35" t="s">
-        <v>144</v>
-      </c>
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
@@ -13653,15 +13031,9 @@
       <c r="O20" s="22"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="C21" s="35" t="s">
-        <v>145</v>
-      </c>
+      <c r="A21" s="22"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
       <c r="D21" s="22"/>
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
@@ -13676,15 +13048,9 @@
       <c r="O21" s="22"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="C22" s="35" t="s">
-        <v>146</v>
-      </c>
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
       <c r="D22" s="22"/>
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
@@ -13699,12 +13065,8 @@
       <c r="O22" s="22"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>148</v>
-      </c>
+      <c r="A23" s="22"/>
+      <c r="B23" s="22"/>
       <c r="C23" s="22"/>
       <c r="D23" s="22"/>
       <c r="E23" s="22"/>
@@ -13720,12 +13082,8 @@
       <c r="O23" s="22"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
-        <v>149</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>89</v>
-      </c>
+      <c r="A24" s="22"/>
+      <c r="B24" s="22"/>
       <c r="C24" s="22"/>
       <c r="D24" s="22"/>
       <c r="E24" s="22"/>
@@ -13741,12 +13099,8 @@
       <c r="O24" s="22"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
-        <v>150</v>
-      </c>
-      <c r="B25" s="35" t="s">
-        <v>151</v>
-      </c>
+      <c r="A25" s="22"/>
+      <c r="B25" s="22"/>
       <c r="C25" s="22"/>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
@@ -14478,12 +13832,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>152</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14502,19 +13856,19 @@
         <v>78</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>155</v>
+        <v>129</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>156</v>
+        <v>130</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>157</v>
+        <v>131</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>158</v>
+        <v>132</v>
       </c>
       <c r="I4" s="19" t="s">
         <v>87</v>
@@ -14540,10 +13894,10 @@
         <v>10</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>159</v>
+        <v>133</v>
       </c>
       <c r="H5" s="24" t="s">
-        <v>160</v>
+        <v>134</v>
       </c>
       <c r="I5" s="26"/>
     </row>
@@ -15648,16 +15002,16 @@
       <c r="I105" s="22"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="36" t="s">
-        <v>161</v>
+      <c r="A108" s="35" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="37" t="s">
-        <v>162</v>
+      <c r="A109" s="36" t="s">
+        <v>136</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="C109" s="5"/>
       <c r="D109" s="5"/>
@@ -15668,11 +15022,11 @@
       <c r="I109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A110" s="37" t="s">
-        <v>164</v>
+      <c r="A110" s="36" t="s">
+        <v>138</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>165</v>
+        <v>139</v>
       </c>
       <c r="C110" s="5"/>
       <c r="D110" s="5"/>
@@ -15683,11 +15037,11 @@
       <c r="I110" s="17"/>
     </row>
     <row r="111" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A111" s="37" t="s">
-        <v>166</v>
+      <c r="A111" s="36" t="s">
+        <v>140</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>167</v>
+        <v>141</v>
       </c>
       <c r="C111" s="4"/>
       <c r="D111" s="4"/>
@@ -15698,11 +15052,11 @@
       <c r="I111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A112" s="37" t="s">
-        <v>168</v>
+      <c r="A112" s="36" t="s">
+        <v>142</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>169</v>
+        <v>143</v>
       </c>
       <c r="C112" s="5"/>
       <c r="D112" s="5"/>
@@ -15759,12 +15113,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>170</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>171</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15774,31 +15128,31 @@
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>172</v>
+        <v>146</v>
       </c>
       <c r="B4" s="19" t="s">
         <v>79</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>173</v>
+        <v>147</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>175</v>
+        <v>149</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
       <c r="G4" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>177</v>
+        <v>151</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>178</v>
+        <v>152</v>
       </c>
       <c r="J4" s="19" t="s">
         <v>87</v>
@@ -15806,30 +15160,30 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>179</v>
+        <v>153</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>180</v>
-      </c>
-      <c r="C5" s="38" t="n">
+        <v>154</v>
+      </c>
+      <c r="C5" s="37" t="n">
         <v>42000</v>
       </c>
-      <c r="D5" s="38" t="n">
+      <c r="D5" s="37" t="n">
         <v>40500</v>
       </c>
-      <c r="E5" s="38" t="n">
+      <c r="E5" s="37" t="n">
         <v>41000</v>
       </c>
-      <c r="F5" s="38" t="n">
+      <c r="F5" s="37" t="n">
         <v>39800</v>
       </c>
       <c r="G5" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="H5" s="38" t="n">
+      <c r="H5" s="37" t="n">
         <v>38000000</v>
       </c>
-      <c r="I5" s="38" t="n">
+      <c r="I5" s="37" t="n">
         <v>5200</v>
       </c>
       <c r="J5" s="26"/>
@@ -15837,721 +15191,721 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22"/>
       <c r="B6" s="22"/>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
       <c r="G6" s="22"/>
-      <c r="H6" s="39"/>
-      <c r="I6" s="39"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
       <c r="J6" s="22"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22"/>
       <c r="B7" s="22"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
       <c r="G7" s="22"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="39"/>
+      <c r="H7" s="38"/>
+      <c r="I7" s="38"/>
       <c r="J7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22"/>
       <c r="B8" s="22"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
       <c r="G8" s="22"/>
-      <c r="H8" s="39"/>
-      <c r="I8" s="39"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
       <c r="J8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22"/>
       <c r="B9" s="22"/>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
       <c r="G9" s="22"/>
-      <c r="H9" s="39"/>
-      <c r="I9" s="39"/>
+      <c r="H9" s="38"/>
+      <c r="I9" s="38"/>
       <c r="J9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
       <c r="G10" s="22"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
       <c r="J10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="38"/>
       <c r="G11" s="22"/>
-      <c r="H11" s="39"/>
-      <c r="I11" s="39"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
       <c r="J11" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22"/>
       <c r="B12" s="22"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
       <c r="G12" s="22"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="38"/>
       <c r="J12" s="22"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="22"/>
       <c r="B13" s="22"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
       <c r="G13" s="22"/>
-      <c r="H13" s="39"/>
-      <c r="I13" s="39"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
       <c r="J13" s="22"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="22"/>
       <c r="B14" s="22"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
       <c r="G14" s="22"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="39"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="38"/>
       <c r="J14" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="22"/>
       <c r="B15" s="22"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
       <c r="G15" s="22"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="39"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="38"/>
       <c r="J15" s="22"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22"/>
       <c r="B16" s="22"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
       <c r="G16" s="22"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="39"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
       <c r="J16" s="22"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22"/>
       <c r="B17" s="22"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
       <c r="G17" s="22"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="39"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
       <c r="J17" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22"/>
       <c r="B18" s="22"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
       <c r="G18" s="22"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="39"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="38"/>
       <c r="J18" s="22"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="38"/>
       <c r="G19" s="22"/>
-      <c r="H19" s="39"/>
-      <c r="I19" s="39"/>
+      <c r="H19" s="38"/>
+      <c r="I19" s="38"/>
       <c r="J19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="38"/>
       <c r="G20" s="22"/>
-      <c r="H20" s="39"/>
-      <c r="I20" s="39"/>
+      <c r="H20" s="38"/>
+      <c r="I20" s="38"/>
       <c r="J20" s="22"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="22"/>
       <c r="B21" s="22"/>
-      <c r="C21" s="39"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="39"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="38"/>
       <c r="G21" s="22"/>
-      <c r="H21" s="39"/>
-      <c r="I21" s="39"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="38"/>
       <c r="J21" s="22"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22"/>
       <c r="B22" s="22"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="39"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
       <c r="G22" s="22"/>
-      <c r="H22" s="39"/>
-      <c r="I22" s="39"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="38"/>
       <c r="J22" s="22"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22"/>
       <c r="B23" s="22"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="38"/>
       <c r="G23" s="22"/>
-      <c r="H23" s="39"/>
-      <c r="I23" s="39"/>
+      <c r="H23" s="38"/>
+      <c r="I23" s="38"/>
       <c r="J23" s="22"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="22"/>
       <c r="B24" s="22"/>
-      <c r="C24" s="39"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
       <c r="G24" s="22"/>
-      <c r="H24" s="39"/>
-      <c r="I24" s="39"/>
+      <c r="H24" s="38"/>
+      <c r="I24" s="38"/>
       <c r="J24" s="22"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22"/>
       <c r="B25" s="22"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
       <c r="G25" s="22"/>
-      <c r="H25" s="39"/>
-      <c r="I25" s="39"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="38"/>
       <c r="J25" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="22"/>
       <c r="B26" s="22"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
       <c r="G26" s="22"/>
-      <c r="H26" s="39"/>
-      <c r="I26" s="39"/>
+      <c r="H26" s="38"/>
+      <c r="I26" s="38"/>
       <c r="J26" s="22"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="22"/>
       <c r="B27" s="22"/>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
       <c r="G27" s="22"/>
-      <c r="H27" s="39"/>
-      <c r="I27" s="39"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="38"/>
       <c r="J27" s="22"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
       <c r="G28" s="22"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="39"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="38"/>
       <c r="J28" s="22"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="22"/>
       <c r="B29" s="22"/>
-      <c r="C29" s="39"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="38"/>
       <c r="G29" s="22"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="39"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="38"/>
       <c r="J29" s="22"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22"/>
       <c r="B30" s="22"/>
-      <c r="C30" s="39"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="38"/>
       <c r="G30" s="22"/>
-      <c r="H30" s="39"/>
-      <c r="I30" s="39"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="38"/>
       <c r="J30" s="22"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="22"/>
       <c r="B31" s="22"/>
-      <c r="C31" s="39"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="39"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="38"/>
       <c r="G31" s="22"/>
-      <c r="H31" s="39"/>
-      <c r="I31" s="39"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="38"/>
       <c r="J31" s="22"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="22"/>
       <c r="B32" s="22"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="39"/>
+      <c r="C32" s="38"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="38"/>
       <c r="G32" s="22"/>
-      <c r="H32" s="39"/>
-      <c r="I32" s="39"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="38"/>
       <c r="J32" s="22"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="22"/>
       <c r="B33" s="22"/>
-      <c r="C33" s="39"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="39"/>
-      <c r="F33" s="39"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
       <c r="G33" s="22"/>
-      <c r="H33" s="39"/>
-      <c r="I33" s="39"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="38"/>
       <c r="J33" s="22"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="22"/>
       <c r="B34" s="22"/>
-      <c r="C34" s="39"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
       <c r="G34" s="22"/>
-      <c r="H34" s="39"/>
-      <c r="I34" s="39"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="38"/>
       <c r="J34" s="22"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="22"/>
       <c r="B35" s="22"/>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="39"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
       <c r="G35" s="22"/>
-      <c r="H35" s="39"/>
-      <c r="I35" s="39"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="38"/>
       <c r="J35" s="22"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="22"/>
       <c r="B36" s="22"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
       <c r="G36" s="22"/>
-      <c r="H36" s="39"/>
-      <c r="I36" s="39"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="38"/>
       <c r="J36" s="22"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22"/>
       <c r="B37" s="22"/>
-      <c r="C37" s="39"/>
-      <c r="D37" s="39"/>
-      <c r="E37" s="39"/>
-      <c r="F37" s="39"/>
+      <c r="C37" s="38"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
       <c r="G37" s="22"/>
-      <c r="H37" s="39"/>
-      <c r="I37" s="39"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="38"/>
       <c r="J37" s="22"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22"/>
       <c r="B38" s="22"/>
-      <c r="C38" s="39"/>
-      <c r="D38" s="39"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="39"/>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
       <c r="G38" s="22"/>
-      <c r="H38" s="39"/>
-      <c r="I38" s="39"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="38"/>
       <c r="J38" s="22"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="22"/>
       <c r="B39" s="22"/>
-      <c r="C39" s="39"/>
-      <c r="D39" s="39"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="39"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="38"/>
       <c r="G39" s="22"/>
-      <c r="H39" s="39"/>
-      <c r="I39" s="39"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="38"/>
       <c r="J39" s="22"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="22"/>
       <c r="B40" s="22"/>
-      <c r="C40" s="39"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="39"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="38"/>
       <c r="G40" s="22"/>
-      <c r="H40" s="39"/>
-      <c r="I40" s="39"/>
+      <c r="H40" s="38"/>
+      <c r="I40" s="38"/>
       <c r="J40" s="22"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="22"/>
       <c r="B41" s="22"/>
-      <c r="C41" s="39"/>
-      <c r="D41" s="39"/>
-      <c r="E41" s="39"/>
-      <c r="F41" s="39"/>
+      <c r="C41" s="38"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="38"/>
       <c r="G41" s="22"/>
-      <c r="H41" s="39"/>
-      <c r="I41" s="39"/>
+      <c r="H41" s="38"/>
+      <c r="I41" s="38"/>
       <c r="J41" s="22"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22"/>
       <c r="B42" s="22"/>
-      <c r="C42" s="39"/>
-      <c r="D42" s="39"/>
-      <c r="E42" s="39"/>
-      <c r="F42" s="39"/>
+      <c r="C42" s="38"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="38"/>
       <c r="G42" s="22"/>
-      <c r="H42" s="39"/>
-      <c r="I42" s="39"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="38"/>
       <c r="J42" s="22"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="22"/>
       <c r="B43" s="22"/>
-      <c r="C43" s="39"/>
-      <c r="D43" s="39"/>
-      <c r="E43" s="39"/>
-      <c r="F43" s="39"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
       <c r="G43" s="22"/>
-      <c r="H43" s="39"/>
-      <c r="I43" s="39"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="38"/>
       <c r="J43" s="22"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="22"/>
       <c r="B44" s="22"/>
-      <c r="C44" s="39"/>
-      <c r="D44" s="39"/>
-      <c r="E44" s="39"/>
-      <c r="F44" s="39"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
       <c r="G44" s="22"/>
-      <c r="H44" s="39"/>
-      <c r="I44" s="39"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="38"/>
       <c r="J44" s="22"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22"/>
       <c r="B45" s="22"/>
-      <c r="C45" s="39"/>
-      <c r="D45" s="39"/>
-      <c r="E45" s="39"/>
-      <c r="F45" s="39"/>
+      <c r="C45" s="38"/>
+      <c r="D45" s="38"/>
+      <c r="E45" s="38"/>
+      <c r="F45" s="38"/>
       <c r="G45" s="22"/>
-      <c r="H45" s="39"/>
-      <c r="I45" s="39"/>
+      <c r="H45" s="38"/>
+      <c r="I45" s="38"/>
       <c r="J45" s="22"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="22"/>
       <c r="B46" s="22"/>
-      <c r="C46" s="39"/>
-      <c r="D46" s="39"/>
-      <c r="E46" s="39"/>
-      <c r="F46" s="39"/>
+      <c r="C46" s="38"/>
+      <c r="D46" s="38"/>
+      <c r="E46" s="38"/>
+      <c r="F46" s="38"/>
       <c r="G46" s="22"/>
-      <c r="H46" s="39"/>
-      <c r="I46" s="39"/>
+      <c r="H46" s="38"/>
+      <c r="I46" s="38"/>
       <c r="J46" s="22"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="22"/>
       <c r="B47" s="22"/>
-      <c r="C47" s="39"/>
-      <c r="D47" s="39"/>
-      <c r="E47" s="39"/>
-      <c r="F47" s="39"/>
+      <c r="C47" s="38"/>
+      <c r="D47" s="38"/>
+      <c r="E47" s="38"/>
+      <c r="F47" s="38"/>
       <c r="G47" s="22"/>
-      <c r="H47" s="39"/>
-      <c r="I47" s="39"/>
+      <c r="H47" s="38"/>
+      <c r="I47" s="38"/>
       <c r="J47" s="22"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="22"/>
       <c r="B48" s="22"/>
-      <c r="C48" s="39"/>
-      <c r="D48" s="39"/>
-      <c r="E48" s="39"/>
-      <c r="F48" s="39"/>
+      <c r="C48" s="38"/>
+      <c r="D48" s="38"/>
+      <c r="E48" s="38"/>
+      <c r="F48" s="38"/>
       <c r="G48" s="22"/>
-      <c r="H48" s="39"/>
-      <c r="I48" s="39"/>
+      <c r="H48" s="38"/>
+      <c r="I48" s="38"/>
       <c r="J48" s="22"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="22"/>
       <c r="B49" s="22"/>
-      <c r="C49" s="39"/>
-      <c r="D49" s="39"/>
-      <c r="E49" s="39"/>
-      <c r="F49" s="39"/>
+      <c r="C49" s="38"/>
+      <c r="D49" s="38"/>
+      <c r="E49" s="38"/>
+      <c r="F49" s="38"/>
       <c r="G49" s="22"/>
-      <c r="H49" s="39"/>
-      <c r="I49" s="39"/>
+      <c r="H49" s="38"/>
+      <c r="I49" s="38"/>
       <c r="J49" s="22"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="22"/>
       <c r="B50" s="22"/>
-      <c r="C50" s="39"/>
-      <c r="D50" s="39"/>
-      <c r="E50" s="39"/>
-      <c r="F50" s="39"/>
+      <c r="C50" s="38"/>
+      <c r="D50" s="38"/>
+      <c r="E50" s="38"/>
+      <c r="F50" s="38"/>
       <c r="G50" s="22"/>
-      <c r="H50" s="39"/>
-      <c r="I50" s="39"/>
+      <c r="H50" s="38"/>
+      <c r="I50" s="38"/>
       <c r="J50" s="22"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="22"/>
       <c r="B51" s="22"/>
-      <c r="C51" s="39"/>
-      <c r="D51" s="39"/>
-      <c r="E51" s="39"/>
-      <c r="F51" s="39"/>
+      <c r="C51" s="38"/>
+      <c r="D51" s="38"/>
+      <c r="E51" s="38"/>
+      <c r="F51" s="38"/>
       <c r="G51" s="22"/>
-      <c r="H51" s="39"/>
-      <c r="I51" s="39"/>
+      <c r="H51" s="38"/>
+      <c r="I51" s="38"/>
       <c r="J51" s="22"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="22"/>
       <c r="B52" s="22"/>
-      <c r="C52" s="39"/>
-      <c r="D52" s="39"/>
-      <c r="E52" s="39"/>
-      <c r="F52" s="39"/>
+      <c r="C52" s="38"/>
+      <c r="D52" s="38"/>
+      <c r="E52" s="38"/>
+      <c r="F52" s="38"/>
       <c r="G52" s="22"/>
-      <c r="H52" s="39"/>
-      <c r="I52" s="39"/>
+      <c r="H52" s="38"/>
+      <c r="I52" s="38"/>
       <c r="J52" s="22"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="22"/>
       <c r="B53" s="22"/>
-      <c r="C53" s="39"/>
-      <c r="D53" s="39"/>
-      <c r="E53" s="39"/>
-      <c r="F53" s="39"/>
+      <c r="C53" s="38"/>
+      <c r="D53" s="38"/>
+      <c r="E53" s="38"/>
+      <c r="F53" s="38"/>
       <c r="G53" s="22"/>
-      <c r="H53" s="39"/>
-      <c r="I53" s="39"/>
+      <c r="H53" s="38"/>
+      <c r="I53" s="38"/>
       <c r="J53" s="22"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="22"/>
       <c r="B54" s="22"/>
-      <c r="C54" s="39"/>
-      <c r="D54" s="39"/>
-      <c r="E54" s="39"/>
-      <c r="F54" s="39"/>
+      <c r="C54" s="38"/>
+      <c r="D54" s="38"/>
+      <c r="E54" s="38"/>
+      <c r="F54" s="38"/>
       <c r="G54" s="22"/>
-      <c r="H54" s="39"/>
-      <c r="I54" s="39"/>
+      <c r="H54" s="38"/>
+      <c r="I54" s="38"/>
       <c r="J54" s="22"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22"/>
       <c r="B55" s="22"/>
-      <c r="C55" s="39"/>
-      <c r="D55" s="39"/>
-      <c r="E55" s="39"/>
-      <c r="F55" s="39"/>
+      <c r="C55" s="38"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="38"/>
+      <c r="F55" s="38"/>
       <c r="G55" s="22"/>
-      <c r="H55" s="39"/>
-      <c r="I55" s="39"/>
+      <c r="H55" s="38"/>
+      <c r="I55" s="38"/>
       <c r="J55" s="22"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="22"/>
       <c r="B56" s="22"/>
-      <c r="C56" s="39"/>
-      <c r="D56" s="39"/>
-      <c r="E56" s="39"/>
-      <c r="F56" s="39"/>
+      <c r="C56" s="38"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="38"/>
+      <c r="F56" s="38"/>
       <c r="G56" s="22"/>
-      <c r="H56" s="39"/>
-      <c r="I56" s="39"/>
+      <c r="H56" s="38"/>
+      <c r="I56" s="38"/>
       <c r="J56" s="22"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="22"/>
       <c r="B57" s="22"/>
-      <c r="C57" s="39"/>
-      <c r="D57" s="39"/>
-      <c r="E57" s="39"/>
-      <c r="F57" s="39"/>
+      <c r="C57" s="38"/>
+      <c r="D57" s="38"/>
+      <c r="E57" s="38"/>
+      <c r="F57" s="38"/>
       <c r="G57" s="22"/>
-      <c r="H57" s="39"/>
-      <c r="I57" s="39"/>
+      <c r="H57" s="38"/>
+      <c r="I57" s="38"/>
       <c r="J57" s="22"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="22"/>
       <c r="B58" s="22"/>
-      <c r="C58" s="39"/>
-      <c r="D58" s="39"/>
-      <c r="E58" s="39"/>
-      <c r="F58" s="39"/>
+      <c r="C58" s="38"/>
+      <c r="D58" s="38"/>
+      <c r="E58" s="38"/>
+      <c r="F58" s="38"/>
       <c r="G58" s="22"/>
-      <c r="H58" s="39"/>
-      <c r="I58" s="39"/>
+      <c r="H58" s="38"/>
+      <c r="I58" s="38"/>
       <c r="J58" s="22"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="22"/>
       <c r="B59" s="22"/>
-      <c r="C59" s="39"/>
-      <c r="D59" s="39"/>
-      <c r="E59" s="39"/>
-      <c r="F59" s="39"/>
+      <c r="C59" s="38"/>
+      <c r="D59" s="38"/>
+      <c r="E59" s="38"/>
+      <c r="F59" s="38"/>
       <c r="G59" s="22"/>
-      <c r="H59" s="39"/>
-      <c r="I59" s="39"/>
+      <c r="H59" s="38"/>
+      <c r="I59" s="38"/>
       <c r="J59" s="22"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="22"/>
       <c r="B60" s="22"/>
-      <c r="C60" s="39"/>
-      <c r="D60" s="39"/>
-      <c r="E60" s="39"/>
-      <c r="F60" s="39"/>
+      <c r="C60" s="38"/>
+      <c r="D60" s="38"/>
+      <c r="E60" s="38"/>
+      <c r="F60" s="38"/>
       <c r="G60" s="22"/>
-      <c r="H60" s="39"/>
-      <c r="I60" s="39"/>
+      <c r="H60" s="38"/>
+      <c r="I60" s="38"/>
       <c r="J60" s="22"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="22"/>
       <c r="B61" s="22"/>
-      <c r="C61" s="39"/>
-      <c r="D61" s="39"/>
-      <c r="E61" s="39"/>
-      <c r="F61" s="39"/>
+      <c r="C61" s="38"/>
+      <c r="D61" s="38"/>
+      <c r="E61" s="38"/>
+      <c r="F61" s="38"/>
       <c r="G61" s="22"/>
-      <c r="H61" s="39"/>
-      <c r="I61" s="39"/>
+      <c r="H61" s="38"/>
+      <c r="I61" s="38"/>
       <c r="J61" s="22"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="22"/>
       <c r="B62" s="22"/>
-      <c r="C62" s="39"/>
-      <c r="D62" s="39"/>
-      <c r="E62" s="39"/>
-      <c r="F62" s="39"/>
+      <c r="C62" s="38"/>
+      <c r="D62" s="38"/>
+      <c r="E62" s="38"/>
+      <c r="F62" s="38"/>
       <c r="G62" s="22"/>
-      <c r="H62" s="39"/>
-      <c r="I62" s="39"/>
+      <c r="H62" s="38"/>
+      <c r="I62" s="38"/>
       <c r="J62" s="22"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="22"/>
       <c r="B63" s="22"/>
-      <c r="C63" s="39"/>
-      <c r="D63" s="39"/>
-      <c r="E63" s="39"/>
-      <c r="F63" s="39"/>
+      <c r="C63" s="38"/>
+      <c r="D63" s="38"/>
+      <c r="E63" s="38"/>
+      <c r="F63" s="38"/>
       <c r="G63" s="22"/>
-      <c r="H63" s="39"/>
-      <c r="I63" s="39"/>
+      <c r="H63" s="38"/>
+      <c r="I63" s="38"/>
       <c r="J63" s="22"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="22"/>
       <c r="B64" s="22"/>
-      <c r="C64" s="39"/>
-      <c r="D64" s="39"/>
-      <c r="E64" s="39"/>
-      <c r="F64" s="39"/>
+      <c r="C64" s="38"/>
+      <c r="D64" s="38"/>
+      <c r="E64" s="38"/>
+      <c r="F64" s="38"/>
       <c r="G64" s="22"/>
-      <c r="H64" s="39"/>
-      <c r="I64" s="39"/>
+      <c r="H64" s="38"/>
+      <c r="I64" s="38"/>
       <c r="J64" s="22"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="22"/>
       <c r="B65" s="22"/>
-      <c r="C65" s="39"/>
-      <c r="D65" s="39"/>
-      <c r="E65" s="39"/>
-      <c r="F65" s="39"/>
+      <c r="C65" s="38"/>
+      <c r="D65" s="38"/>
+      <c r="E65" s="38"/>
+      <c r="F65" s="38"/>
       <c r="G65" s="22"/>
-      <c r="H65" s="39"/>
-      <c r="I65" s="39"/>
+      <c r="H65" s="38"/>
+      <c r="I65" s="38"/>
       <c r="J65" s="22"/>
     </row>
   </sheetData>
@@ -16593,12 +15947,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>181</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>182</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16629,7 +15983,7 @@
         <v>14</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="I4" s="19" t="s">
         <v>87</v>
@@ -16655,13 +16009,13 @@
         <v>93</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>184</v>
+        <v>158</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>45</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>185</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17808,12 +17162,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>187</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17823,39 +17177,39 @@
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>188</v>
+        <v>162</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>189</v>
+        <v>163</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>190</v>
+        <v>164</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>191</v>
+        <v>165</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>192</v>
+        <v>166</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>193</v>
+        <v>167</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>194</v>
+        <v>168</v>
       </c>
       <c r="H4" s="19" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35" t="s">
-        <v>195</v>
+      <c r="A5" s="39" t="s">
+        <v>169</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="C5" s="35" t="s">
-        <v>196</v>
+        <v>170</v>
+      </c>
+      <c r="C5" s="39" t="s">
+        <v>171</v>
       </c>
       <c r="D5" s="22"/>
       <c r="E5" s="22"/>
@@ -17864,14 +17218,14 @@
       <c r="H5" s="22"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="35" t="s">
-        <v>197</v>
+      <c r="A6" s="39" t="s">
+        <v>172</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="C6" s="35" t="s">
-        <v>198</v>
+        <v>170</v>
+      </c>
+      <c r="C6" s="39" t="s">
+        <v>173</v>
       </c>
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
@@ -17880,14 +17234,14 @@
       <c r="H6" s="22"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="35" t="s">
-        <v>199</v>
+      <c r="A7" s="39" t="s">
+        <v>174</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>200</v>
-      </c>
-      <c r="C7" s="35" t="s">
-        <v>201</v>
+        <v>175</v>
+      </c>
+      <c r="C7" s="39" t="s">
+        <v>176</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
@@ -17896,14 +17250,14 @@
       <c r="H7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="s">
-        <v>202</v>
+      <c r="A8" s="39" t="s">
+        <v>177</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>200</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>201</v>
+        <v>175</v>
+      </c>
+      <c r="C8" s="39" t="s">
+        <v>176</v>
       </c>
       <c r="D8" s="22"/>
       <c r="E8" s="22"/>
@@ -17912,14 +17266,14 @@
       <c r="H8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="35" t="s">
-        <v>203</v>
+      <c r="A9" s="39" t="s">
+        <v>178</v>
       </c>
       <c r="B9" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="C9" s="35" t="s">
-        <v>204</v>
+      <c r="C9" s="39" t="s">
+        <v>179</v>
       </c>
       <c r="D9" s="22"/>
       <c r="E9" s="22"/>
@@ -17928,14 +17282,14 @@
       <c r="H9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="35" t="s">
-        <v>205</v>
+      <c r="A10" s="39" t="s">
+        <v>180</v>
       </c>
       <c r="B10" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="C10" s="35" t="s">
-        <v>206</v>
+      <c r="C10" s="39" t="s">
+        <v>181</v>
       </c>
       <c r="D10" s="22"/>
       <c r="E10" s="22"/>
@@ -17944,14 +17298,14 @@
       <c r="H10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="35" t="s">
-        <v>207</v>
+      <c r="A11" s="39" t="s">
+        <v>182</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="C11" s="35" t="s">
-        <v>208</v>
+        <v>183</v>
+      </c>
+      <c r="C11" s="39" t="s">
+        <v>184</v>
       </c>
       <c r="D11" s="22"/>
       <c r="E11" s="22"/>
@@ -17960,14 +17314,14 @@
       <c r="H11" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="35" t="s">
-        <v>209</v>
+      <c r="A12" s="39" t="s">
+        <v>185</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="C12" s="35" t="s">
-        <v>208</v>
+        <v>183</v>
+      </c>
+      <c r="C12" s="39" t="s">
+        <v>184</v>
       </c>
       <c r="D12" s="22"/>
       <c r="E12" s="22"/>
@@ -17976,14 +17330,14 @@
       <c r="H12" s="22"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="B13" s="35" t="s">
-        <v>151</v>
-      </c>
-      <c r="C13" s="35" t="s">
-        <v>211</v>
+      <c r="A13" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="B13" s="39" t="s">
+        <v>187</v>
+      </c>
+      <c r="C13" s="39" t="s">
+        <v>188</v>
       </c>
       <c r="D13" s="22"/>
       <c r="E13" s="22"/>
@@ -17992,14 +17346,14 @@
       <c r="H13" s="22"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="35" t="s">
-        <v>212</v>
-      </c>
-      <c r="B14" s="35" t="s">
-        <v>151</v>
-      </c>
-      <c r="C14" s="35" t="s">
-        <v>211</v>
+      <c r="A14" s="39" t="s">
+        <v>189</v>
+      </c>
+      <c r="B14" s="39" t="s">
+        <v>187</v>
+      </c>
+      <c r="C14" s="39" t="s">
+        <v>188</v>
       </c>
       <c r="D14" s="22"/>
       <c r="E14" s="22"/>
@@ -18008,14 +17362,14 @@
       <c r="H14" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="35" t="s">
-        <v>213</v>
+      <c r="A15" s="39" t="s">
+        <v>190</v>
       </c>
       <c r="B15" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="C15" s="35" t="s">
-        <v>214</v>
+      <c r="C15" s="39" t="s">
+        <v>191</v>
       </c>
       <c r="D15" s="22"/>
       <c r="E15" s="22"/>
@@ -18024,14 +17378,14 @@
       <c r="H15" s="22"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="35" t="s">
-        <v>215</v>
+      <c r="A16" s="39" t="s">
+        <v>192</v>
       </c>
       <c r="B16" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="C16" s="35" t="s">
-        <v>214</v>
+      <c r="C16" s="39" t="s">
+        <v>191</v>
       </c>
       <c r="D16" s="22"/>
       <c r="E16" s="22"/>
@@ -18040,14 +17394,14 @@
       <c r="H16" s="22"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="35" t="s">
-        <v>216</v>
+      <c r="A17" s="39" t="s">
+        <v>193</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>217</v>
-      </c>
-      <c r="C17" s="35" t="s">
-        <v>218</v>
+        <v>194</v>
+      </c>
+      <c r="C17" s="39" t="s">
+        <v>195</v>
       </c>
       <c r="D17" s="22"/>
       <c r="E17" s="22"/>
@@ -18056,14 +17410,14 @@
       <c r="H17" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="35" t="s">
-        <v>219</v>
+      <c r="A18" s="39" t="s">
+        <v>196</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>217</v>
-      </c>
-      <c r="C18" s="35" t="s">
-        <v>220</v>
+        <v>194</v>
+      </c>
+      <c r="C18" s="39" t="s">
+        <v>197</v>
       </c>
       <c r="D18" s="22"/>
       <c r="E18" s="22"/>
@@ -18072,14 +17426,14 @@
       <c r="H18" s="22"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="35" t="s">
-        <v>221</v>
+      <c r="A19" s="39" t="s">
+        <v>198</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>217</v>
-      </c>
-      <c r="C19" s="35" t="s">
-        <v>222</v>
+        <v>194</v>
+      </c>
+      <c r="C19" s="39" t="s">
+        <v>199</v>
       </c>
       <c r="D19" s="22"/>
       <c r="E19" s="22"/>
@@ -18088,14 +17442,14 @@
       <c r="H19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="35" t="s">
-        <v>223</v>
+      <c r="A20" s="39" t="s">
+        <v>200</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>224</v>
-      </c>
-      <c r="C20" s="35" t="s">
-        <v>225</v>
+        <v>201</v>
+      </c>
+      <c r="C20" s="39" t="s">
+        <v>202</v>
       </c>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
@@ -18104,14 +17458,14 @@
       <c r="H20" s="22"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="35" t="s">
-        <v>226</v>
+      <c r="A21" s="39" t="s">
+        <v>203</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>224</v>
-      </c>
-      <c r="C21" s="35" t="s">
-        <v>225</v>
+        <v>201</v>
+      </c>
+      <c r="C21" s="39" t="s">
+        <v>202</v>
       </c>
       <c r="D21" s="22"/>
       <c r="E21" s="22"/>
@@ -18120,14 +17474,14 @@
       <c r="H21" s="22"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="35" t="s">
-        <v>227</v>
+      <c r="A22" s="39" t="s">
+        <v>204</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>228</v>
-      </c>
-      <c r="C22" s="35" t="s">
-        <v>229</v>
+        <v>205</v>
+      </c>
+      <c r="C22" s="39" t="s">
+        <v>206</v>
       </c>
       <c r="D22" s="22"/>
       <c r="E22" s="22"/>

</xml_diff>